<commit_message>
Updated Testing Matrix and Timeline
</commit_message>
<xml_diff>
--- a/GAM-305TestingMatrix.xlsx
+++ b/GAM-305TestingMatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\irnin\Documents\Unreal Projects\GAM305Final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BEF0FD-A395-46E4-92AC-916593146A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB3E3AF-0B99-4B16-9A5A-87A1604AC14A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24975" yWindow="2355" windowWidth="27075" windowHeight="14925" xr2:uid="{19EF330C-6F54-4365-A47E-10806019DE9B}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{19EF330C-6F54-4365-A47E-10806019DE9B}"/>
   </bookViews>
   <sheets>
     <sheet name="Traceability Matrix" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
   <si>
     <t>Traceability Matrix</t>
   </si>
@@ -123,30 +123,6 @@
     <t>Level</t>
   </si>
   <si>
-    <t>Player Character basics</t>
-  </si>
-  <si>
-    <t>Player Character Health and Death</t>
-  </si>
-  <si>
-    <t>Pickup</t>
-  </si>
-  <si>
-    <t>Player Character moves around and attacks</t>
-  </si>
-  <si>
-    <t>Player Character displays health and dies when health reaches zero</t>
-  </si>
-  <si>
-    <t>Enemies track the player and attacks</t>
-  </si>
-  <si>
-    <t>Player can pick up equipment and power ups</t>
-  </si>
-  <si>
-    <t>Player can move around the level and cannot get out of bounds</t>
-  </si>
-  <si>
     <t>Mason France</t>
   </si>
   <si>
@@ -156,7 +132,61 @@
     <t>Ranged Attack with a bow and arrow, Melee Attack with a sword.</t>
   </si>
   <si>
-    <t>Player uses WASD to move around.</t>
+    <t>Rusty Lewis</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Player Character Movement</t>
+  </si>
+  <si>
+    <t>Player Character moves using WASD</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>No bugs reported</t>
+  </si>
+  <si>
+    <t>Player Character Mouse Following</t>
+  </si>
+  <si>
+    <t>Player Character follows the mouse cursor</t>
+  </si>
+  <si>
+    <t>Bow Enemy Follows Player</t>
+  </si>
+  <si>
+    <t>Bow enemy successfully follows the character and loses sight after a certain distance</t>
+  </si>
+  <si>
+    <t>Bow enemy would not lose the player after a certain distance</t>
+  </si>
+  <si>
+    <t>Bugs Fixed?</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Mortar Enemy Follows Player</t>
+  </si>
+  <si>
+    <t>Mortar enemy successfully follows the character and loses sight after a certain distance</t>
+  </si>
+  <si>
+    <t>Christopher Rockwell</t>
+  </si>
+  <si>
+    <t>Kylan Konopaski</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Player uses WASD to move around, Character follows Mouse Cursor</t>
   </si>
 </sst>
 </file>
@@ -456,6 +486,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -473,37 +527,83 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="11">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -867,32 +967,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
     </row>
     <row r="2" spans="1:22" s="4" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="34"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="28"/>
       <c r="J2" s="13"/>
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
@@ -911,16 +1011,16 @@
       <c r="A3" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="38"/>
-      <c r="H3" s="38"/>
-      <c r="I3" s="39"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="33"/>
     </row>
     <row r="4" spans="1:22" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
@@ -967,10 +1067,13 @@
         <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="I6" s="15"/>
     </row>
@@ -979,7 +1082,10 @@
         <v>19</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>30</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>23</v>
@@ -1000,10 +1106,10 @@
         <v>21</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>23</v>
@@ -1014,6 +1120,9 @@
       <c r="B10" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="E10" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="F10" s="1" t="s">
         <v>23</v>
       </c>
@@ -1023,23 +1132,44 @@
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="F11" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I11" s="15"/>
     </row>
     <row r="12" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="E12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I12" s="15"/>
     </row>
     <row r="13" spans="1:22" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="E13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>23</v>
+      </c>
       <c r="I13" s="15"/>
     </row>
     <row r="14" spans="1:22" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>27</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="I14" s="15"/>
     </row>
@@ -1143,10 +1273,10 @@
     <mergeCell ref="B3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="F5:F38">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1160,7 +1290,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748CED0D-D7CE-4618-A56E-B7666AE2995E}">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
@@ -1173,26 +1303,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="28"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="36"/>
     </row>
     <row r="2" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="37" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="31"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="3" spans="1:7" s="8" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -1207,65 +1337,81 @@
       <c r="D3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="6" t="s">
+        <v>42</v>
+      </c>
       <c r="F3" s="6"/>
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7" ht="93.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="9"/>
     </row>
     <row r="5" spans="1:7" ht="111" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="15"/>
+      <c r="A5" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:7" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+        <v>40</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="F6" s="15"/>
     </row>
     <row r="7" spans="1:7" ht="97.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+        <v>45</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="E7" s="1"/>
       <c r="F7" s="15"/>
     </row>
     <row r="8" spans="1:7" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>35</v>
-      </c>
+      <c r="A8" s="25"/>
+      <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1512,8 +1658,12 @@
       <c r="F38" s="15"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="12"/>
-      <c r="F39" s="10"/>
+      <c r="A39" s="25"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="15"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="12"/>
@@ -1550,18 +1700,30 @@
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12"/>
       <c r="F48" s="10"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="12"/>
+      <c r="F49" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B2:F2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4:C22">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="C4:C23">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4:E29">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>"Pass"</formula>
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -1584,15 +1746,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003FC679AA94041F4BA4494D199A3447AF" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7f196c085cfdbd30e0a6b7617037a918">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382" xmlns:ns3="f716dd8a-49a0-4c40-b209-038e1651b548" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c32ca31bb9a34b5b0e8feded347fb44b" ns2:_="" ns3:_="">
     <xsd:import namespace="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382"/>
@@ -1849,6 +2002,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F271AB-EFB2-4823-A2F0-9F2289E658DB}">
   <ds:schemaRefs>
@@ -1863,14 +2025,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81B87576-EBB2-43B7-B881-33A6175934F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1887,4 +2041,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>